<commit_message>
v1.13.0 - Treinos reativado: um card por treino + peso e observacoes
- Pagina Treinos cria um card por treino (titulo definido na planilha; fallback Treino A/B/C)
- Execucao mostra series x reps, descanso, campo de peso ao lado e observacoes abaixo
- Peso salvo por exercicio no aparelho
- Leitor entende linhas de titulo (Tipo "-") e agrupa por treino

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eltech_personality_modelo.xlsx
+++ b/eltech_personality_modelo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imgoffice-my.sharepoint.com/personal/salatiel_ferreira_img_com_br/Documents/Desktop/Documentos/PERSONALITY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="332" documentId="11_2F4EA715163889BF4D052CB0C8F7AF26202D6828" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2897BB43-1162-44F6-BE4D-B955B006F9E7}"/>
+  <xr:revisionPtr revIDLastSave="389" documentId="11_2F4EA715163889BF4D052CB0C8F7AF26202D6828" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{162CCF8C-92F4-4463-968C-A88F5CCDD95D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="119">
   <si>
     <t/>
   </si>
@@ -348,6 +348,36 @@
   </si>
   <si>
     <t>OBSERVAÇÃO</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>PANTURRILHA</t>
+  </si>
+  <si>
+    <t>DESENVOLVIMENTO</t>
+  </si>
+  <si>
+    <t>ELEVAÇÃO FRONTA</t>
+  </si>
+  <si>
+    <t>TRAPEZIO</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>10 - 12</t>
+  </si>
+  <si>
+    <t>TREINO 1</t>
+  </si>
+  <si>
+    <t>TREINO 2</t>
+  </si>
+  <si>
+    <t>TESTE</t>
   </si>
 </sst>
 </file>
@@ -460,7 +490,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -498,13 +528,22 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -859,16 +898,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="14"/>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
+      <c r="A2" s="18"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1635,33 +1674,35 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.69921875" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.69921875" style="5" customWidth="1"/>
-    <col min="3" max="5" width="15.69921875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="15.69921875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.69921875" style="13" customWidth="1"/>
+    <col min="5" max="5" width="15.69921875" style="1" customWidth="1"/>
     <col min="6" max="6" width="15.69921875" customWidth="1"/>
     <col min="7" max="7" width="8.796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="13"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="A2" s="16"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1674,7 +1715,7 @@
       <c r="C4" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="14" t="s">
         <v>89</v>
       </c>
       <c r="E4" s="12" t="s">
@@ -1685,20 +1726,23 @@
       </c>
     </row>
     <row r="5" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="1">
-        <v>4</v>
-      </c>
-      <c r="D5" s="1">
-        <v>10</v>
-      </c>
-      <c r="E5" s="1">
-        <v>60</v>
+      <c r="A5" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1706,13 +1750,13 @@
         <v>73</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" s="1">
         <v>4</v>
       </c>
-      <c r="D6" s="1">
-        <v>10</v>
+      <c r="D6" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="E6" s="1">
         <v>60</v>
@@ -1723,13 +1767,13 @@
         <v>73</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C7" s="1">
         <v>4</v>
       </c>
-      <c r="D7" s="1">
-        <v>10</v>
+      <c r="D7" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="E7" s="1">
         <v>60</v>
@@ -1740,13 +1784,13 @@
         <v>73</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C8" s="1">
         <v>4</v>
       </c>
-      <c r="D8" s="1">
-        <v>10</v>
+      <c r="D8" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="E8" s="1">
         <v>60</v>
@@ -1757,13 +1801,13 @@
         <v>73</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C9" s="1">
         <v>4</v>
       </c>
-      <c r="D9" s="1">
-        <v>10</v>
+      <c r="D9" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="E9" s="1">
         <v>60</v>
@@ -1771,36 +1815,39 @@
     </row>
     <row r="10" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C10" s="1">
-        <v>3</v>
-      </c>
-      <c r="D10" s="1">
-        <v>12</v>
+        <v>4</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>115</v>
       </c>
       <c r="E10" s="1">
         <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C11" s="1">
-        <v>3</v>
-      </c>
-      <c r="D11" s="1">
-        <v>12</v>
-      </c>
-      <c r="E11" s="1">
-        <v>60</v>
+      <c r="A11" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1808,12 +1855,12 @@
         <v>74</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C12" s="1">
         <v>3</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="13">
         <v>12</v>
       </c>
       <c r="E12" s="1">
@@ -1825,22 +1872,16 @@
         <v>74</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C13" s="1">
         <v>3</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="13">
         <v>12</v>
       </c>
       <c r="E13" s="1">
         <v>60</v>
-      </c>
-      <c r="F13" t="s">
-        <v>0</v>
-      </c>
-      <c r="G13" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1848,36 +1889,30 @@
         <v>74</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C14" s="1">
         <v>3</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="13">
         <v>12</v>
       </c>
       <c r="E14" s="1">
         <v>60</v>
       </c>
-      <c r="F14" t="s">
-        <v>0</v>
-      </c>
-      <c r="G14" t="s">
-        <v>0</v>
-      </c>
     </row>
     <row r="15" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C15" s="1">
-        <v>4</v>
-      </c>
-      <c r="D15" s="1">
-        <v>15</v>
+        <v>3</v>
+      </c>
+      <c r="D15" s="13">
+        <v>12</v>
       </c>
       <c r="E15" s="1">
         <v>60</v>
@@ -1891,16 +1926,16 @@
     </row>
     <row r="16" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C16" s="1">
-        <v>4</v>
-      </c>
-      <c r="D16" s="1">
-        <v>15</v>
+        <v>3</v>
+      </c>
+      <c r="D16" s="13">
+        <v>12</v>
       </c>
       <c r="E16" s="1">
         <v>60</v>
@@ -1913,26 +1948,23 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C17" s="1">
-        <v>4</v>
-      </c>
-      <c r="D17" s="1">
-        <v>15</v>
-      </c>
-      <c r="E17" s="1">
-        <v>60</v>
-      </c>
-      <c r="F17" t="s">
-        <v>0</v>
-      </c>
-      <c r="G17" t="s">
-        <v>0</v>
+      <c r="A17" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1940,12 +1972,12 @@
         <v>75</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C18" s="1">
         <v>4</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="13">
         <v>15</v>
       </c>
       <c r="E18" s="1">
@@ -1963,12 +1995,12 @@
         <v>75</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C19" s="1">
         <v>4</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="13">
         <v>15</v>
       </c>
       <c r="E19" s="1">
@@ -1982,14 +2014,20 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>0</v>
+      <c r="A20" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" s="1">
+        <v>4</v>
+      </c>
+      <c r="D20" s="13">
+        <v>15</v>
+      </c>
+      <c r="E20" s="1">
+        <v>60</v>
       </c>
       <c r="F20" t="s">
         <v>0</v>
@@ -1999,14 +2037,20 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>0</v>
+      <c r="A21" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C21" s="1">
+        <v>4</v>
+      </c>
+      <c r="D21" s="13">
+        <v>15</v>
+      </c>
+      <c r="E21" s="1">
+        <v>60</v>
       </c>
       <c r="F21" t="s">
         <v>0</v>
@@ -2016,14 +2060,20 @@
       </c>
     </row>
     <row r="22" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>0</v>
+      <c r="A22" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" s="1">
+        <v>4</v>
+      </c>
+      <c r="D22" s="13">
+        <v>15</v>
+      </c>
+      <c r="E22" s="1">
+        <v>60</v>
       </c>
       <c r="F22" t="s">
         <v>0</v>
@@ -2033,31 +2083,40 @@
       </c>
     </row>
     <row r="23" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F23" t="s">
-        <v>0</v>
-      </c>
-      <c r="G23" t="s">
-        <v>0</v>
+      <c r="A23" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C24" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>0</v>
+      <c r="A24" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="1">
+        <v>2</v>
+      </c>
+      <c r="D24" s="13">
+        <v>20</v>
+      </c>
+      <c r="E24" s="1">
+        <v>60</v>
       </c>
       <c r="F24" t="s">
         <v>0</v>
@@ -2067,14 +2126,20 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C25" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>0</v>
+      <c r="A25" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C25" s="1">
+        <v>2</v>
+      </c>
+      <c r="D25" s="13">
+        <v>20</v>
+      </c>
+      <c r="E25" s="1">
+        <v>60</v>
       </c>
       <c r="F25" t="s">
         <v>0</v>
@@ -2084,14 +2149,20 @@
       </c>
     </row>
     <row r="26" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C26" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>0</v>
+      <c r="A26" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C26" s="1">
+        <v>2</v>
+      </c>
+      <c r="D26" s="13">
+        <v>20</v>
+      </c>
+      <c r="E26" s="1">
+        <v>60</v>
       </c>
       <c r="F26" t="s">
         <v>0</v>
@@ -2101,14 +2172,20 @@
       </c>
     </row>
     <row r="27" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C27" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>0</v>
+      <c r="A27" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C27" s="1">
+        <v>2</v>
+      </c>
+      <c r="D27" s="13">
+        <v>20</v>
+      </c>
+      <c r="E27" s="1">
+        <v>60</v>
       </c>
       <c r="F27" t="s">
         <v>0</v>
@@ -2121,7 +2198,7 @@
       <c r="C28" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="13" t="s">
         <v>0</v>
       </c>
       <c r="E28" s="1" t="s">
@@ -2138,7 +2215,7 @@
       <c r="C29" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="13" t="s">
         <v>0</v>
       </c>
       <c r="E29" s="1" t="s">
@@ -2155,7 +2232,7 @@
       <c r="C30" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="13" t="s">
         <v>0</v>
       </c>
       <c r="E30" s="1" t="s">
@@ -2172,7 +2249,7 @@
       <c r="C31" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" s="13" t="s">
         <v>0</v>
       </c>
       <c r="E31" s="1" t="s">
@@ -2186,7 +2263,10 @@
       </c>
     </row>
     <row r="32" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D32" s="1" t="s">
+      <c r="C32" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D32" s="13" t="s">
         <v>0</v>
       </c>
       <c r="E32" s="1" t="s">
@@ -2196,6 +2276,71 @@
         <v>0</v>
       </c>
       <c r="G32" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="3:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C33" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D33" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F33" t="s">
+        <v>0</v>
+      </c>
+      <c r="G33" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="3:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C34" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F34" t="s">
+        <v>0</v>
+      </c>
+      <c r="G34" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="3:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C35" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F35" t="s">
+        <v>0</v>
+      </c>
+      <c r="G35" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="3:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D36" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F36" t="s">
+        <v>0</v>
+      </c>
+      <c r="G36" t="s">
         <v>0</v>
       </c>
     </row>
@@ -2205,7 +2350,7 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="C20:C31 D20:G32 F13:G13 F14:G14 F15:G15 F16:G16 F17:G17 F18:G18 F19:G19" numberStoredAsText="1"/>
+    <ignoredError sqref="C28:C35 D28:G36 F15:G15 F16:G16 F18:G18 F19:G19 F20:G20 F21:G21 F22:G22 F24:G24 F25:G25 F26:G26 F27:G27" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
v1.14.4 - Area do Professor sem botoes de remover (troca via importar)
- Removidos "Remover treino" e "Remover ficha"; substituicao acontece ao importar novo .xlsx

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eltech_personality_modelo.xlsx
+++ b/eltech_personality_modelo.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imgoffice-my.sharepoint.com/personal/salatiel_ferreira_img_com_br/Documents/Desktop/Documentos/PERSONALITY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="11_4759A7175C30C5E875C5AEAD6474A9E3A064ACB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8ABA2B58-72F4-4257-AF76-505418789D16}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="11_4759A7175C30C5E875C5AEAD6474A9E3A064ACB4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8693A24-F93C-482D-873B-7C93D3E3226C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ficha do Aluno" sheetId="1" r:id="rId1"/>
     <sheet name="Treino" sheetId="2" r:id="rId2"/>
-    <sheet name="Instruções" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="138">
   <si>
     <t>FICHA DO ALUNO — ELTECH Personality</t>
   </si>
@@ -355,60 +354,6 @@
     <t>Crossover</t>
   </si>
   <si>
-    <t>COMO PREENCHER — ELTECH Personality</t>
-  </si>
-  <si>
-    <t>Este único arquivo alimenta o app do aluno. Preencha as abas 'Ficha do Aluno' e 'Treino'.</t>
-  </si>
-  <si>
-    <t>ABA 'FICHA DO ALUNO'</t>
-  </si>
-  <si>
-    <t>• Não altere os nomes dos campos (coluna da esquerda).</t>
-  </si>
-  <si>
-    <t>• Campos deixados em branco NÃO aparecem no app.</t>
-  </si>
-  <si>
-    <t>• OBJETIVOS: escreva X (ou Sim) nos objetivos desejados.</t>
-  </si>
-  <si>
-    <t>• HISTÓRICO DE SAÚDE: escreva SIM ou NÃO e detalhe na coluna Descrição.</t>
-  </si>
-  <si>
-    <t>• HÁBITOS DE VIDA: escreva a informação na coluna Descrição.</t>
-  </si>
-  <si>
-    <t>• Altura em metros (m); circunferências em cm; dobras cutâneas em mm.</t>
-  </si>
-  <si>
-    <t>• Datas no formato dd/mm/aaaa.</t>
-  </si>
-  <si>
-    <t>ABA 'TREINO'</t>
-  </si>
-  <si>
-    <t>• Colunas: Tipo | Exercício | Séries | Repetições | Descanso | Observação.</t>
-  </si>
-  <si>
-    <t>• TIPO é livre: use o que quiser (A, B, C, Peito, Perna, Segunda...).</t>
-  </si>
-  <si>
-    <t>• Uma linha por exercício, agrupados pelo Tipo.</t>
-  </si>
-  <si>
-    <t>• Repetições pode ser um número (10) ou uma faixa (10-12). Descanso em segundos.</t>
-  </si>
-  <si>
-    <t>• Observação: recado opcional para o aluno naquele exercício.</t>
-  </si>
-  <si>
-    <t>• Vídeo: cole o link do YouTube do exercício (opcional; abre no app com internet).</t>
-  </si>
-  <si>
-    <t>Depois é só enviar o arquivo ao aluno. Ele importa em: Perfil &gt; Área do Professor &gt; Importar dados.</t>
-  </si>
-  <si>
     <t>https://www.youtube.com/watch?v=LT_nelifZ_k</t>
   </si>
   <si>
@@ -440,16 +385,87 @@
   </si>
   <si>
     <t>15 - 20</t>
+  </si>
+  <si>
+    <t>Salatiel</t>
+  </si>
+  <si>
+    <t>1.82</t>
+  </si>
+  <si>
+    <t>Mascolino</t>
+  </si>
+  <si>
+    <t>(12)982650263</t>
+  </si>
+  <si>
+    <t>saala.eng@gmail.com</t>
+  </si>
+  <si>
+    <t>Desenvolvedor</t>
+  </si>
+  <si>
+    <t>(12)997182612</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>NÃO</t>
+  </si>
+  <si>
+    <t>SIM</t>
+  </si>
+  <si>
+    <t>Rompimento do tecido muscular do biceps esquerdo</t>
+  </si>
+  <si>
+    <t>Uma vez ao dia</t>
+  </si>
+  <si>
+    <t>Musculação</t>
+  </si>
+  <si>
+    <t>1h</t>
+  </si>
+  <si>
+    <t>5h</t>
+  </si>
+  <si>
+    <t>4 Litros por dia</t>
+  </si>
+  <si>
+    <t>Ruim</t>
+  </si>
+  <si>
+    <t>Sociavel</t>
+  </si>
+  <si>
+    <t>Não</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Intermediaria</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -472,13 +488,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -859,7 +879,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>117</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
@@ -869,8 +889,8 @@
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
-        <v>7</v>
+      <c r="B7">
+        <v>22</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
@@ -881,7 +901,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>118</v>
       </c>
       <c r="C8" t="s">
         <v>11</v>
@@ -891,8 +911,8 @@
       <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s">
-        <v>7</v>
+      <c r="B9">
+        <v>100</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
@@ -903,7 +923,7 @@
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -913,8 +933,8 @@
       <c r="A11" t="s">
         <v>15</v>
       </c>
-      <c r="B11" t="s">
-        <v>7</v>
+      <c r="B11" s="1">
+        <v>45633</v>
       </c>
       <c r="C11" t="s">
         <v>7</v>
@@ -925,7 +945,7 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>7</v>
+        <v>120</v>
       </c>
       <c r="C12" t="s">
         <v>7</v>
@@ -935,8 +955,8 @@
       <c r="A13" t="s">
         <v>17</v>
       </c>
-      <c r="B13" t="s">
-        <v>7</v>
+      <c r="B13" s="2" t="s">
+        <v>121</v>
       </c>
       <c r="C13" t="s">
         <v>7</v>
@@ -947,7 +967,7 @@
         <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>7</v>
+        <v>122</v>
       </c>
       <c r="C14" t="s">
         <v>7</v>
@@ -958,7 +978,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>7</v>
+        <v>123</v>
       </c>
       <c r="C15" t="s">
         <v>7</v>
@@ -982,7 +1002,7 @@
         <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>7</v>
+        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -990,7 +1010,7 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>7</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -998,7 +1018,7 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>7</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -1030,7 +1050,7 @@
         <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>7</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -1054,7 +1074,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>7</v>
+        <v>125</v>
       </c>
       <c r="C29" t="s">
         <v>7</v>
@@ -1065,7 +1085,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>7</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s">
         <v>7</v>
@@ -1076,10 +1096,10 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>7</v>
+        <v>126</v>
       </c>
       <c r="C31" t="s">
-        <v>7</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -1087,7 +1107,7 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>7</v>
+        <v>125</v>
       </c>
       <c r="C32" t="s">
         <v>7</v>
@@ -1098,7 +1118,7 @@
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>7</v>
+        <v>125</v>
       </c>
       <c r="C33" t="s">
         <v>7</v>
@@ -1109,7 +1129,7 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>7</v>
+        <v>125</v>
       </c>
       <c r="C34" t="s">
         <v>7</v>
@@ -1133,7 +1153,7 @@
         <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>7</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -1141,7 +1161,7 @@
         <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>7</v>
+        <v>129</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -1149,7 +1169,7 @@
         <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>7</v>
+        <v>130</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -1157,7 +1177,7 @@
         <v>43</v>
       </c>
       <c r="B41" t="s">
-        <v>7</v>
+        <v>131</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -1165,7 +1185,7 @@
         <v>44</v>
       </c>
       <c r="B42" t="s">
-        <v>7</v>
+        <v>133</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -1173,7 +1193,7 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>7</v>
+        <v>132</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -1181,7 +1201,7 @@
         <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>7</v>
+        <v>134</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -1189,7 +1209,7 @@
         <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>7</v>
+        <v>135</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -1197,7 +1217,7 @@
         <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>7</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -1205,7 +1225,7 @@
         <v>49</v>
       </c>
       <c r="B47" t="s">
-        <v>7</v>
+        <v>137</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -1548,9 +1568,12 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B13" r:id="rId1" xr:uid="{410239A4-F838-4E61-843A-72FC7A275360}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C82" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C5 A16:C18 A6 C6 A7 C7 A8 C8 A9 C9 A10 C10 A11 C11 A12 C12 A13 C13 A14 C14 A15 C15 A22:C24 A19 C19 A20 C20 A21 C21 A26:C28 A25 C25 A35:C37 A29 C29 A30 C30 A31 A32 C32 A33 C33 A34 C34 A48:C82 A38 C38 A39 C39 A40 C40 A41 C41 A42 C42 A43 C43 A44 C44 A45 C45 A46 C46 A47 C47" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1602,7 +1625,7 @@
         <v>92</v>
       </c>
       <c r="B4" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="C4" t="s">
         <v>92</v>
@@ -1640,7 +1663,7 @@
         <v>7</v>
       </c>
       <c r="G5" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1663,7 +1686,7 @@
         <v>7</v>
       </c>
       <c r="G6" t="s">
-        <v>7</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -1686,7 +1709,7 @@
         <v>7</v>
       </c>
       <c r="G7" t="s">
-        <v>7</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -1694,7 +1717,7 @@
         <v>92</v>
       </c>
       <c r="B8" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="C8" t="s">
         <v>92</v>
@@ -1732,7 +1755,7 @@
         <v>7</v>
       </c>
       <c r="G9" t="s">
-        <v>7</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -1755,7 +1778,7 @@
         <v>7</v>
       </c>
       <c r="G10" t="s">
-        <v>7</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -1763,7 +1786,7 @@
         <v>92</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="C11" t="s">
         <v>92</v>
@@ -1801,7 +1824,7 @@
         <v>7</v>
       </c>
       <c r="G12" t="s">
-        <v>7</v>
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -1824,7 +1847,7 @@
         <v>7</v>
       </c>
       <c r="G13" t="s">
-        <v>7</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1832,7 +1855,7 @@
         <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="C14" t="s">
         <v>92</v>
@@ -1852,214 +1875,88 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="B15" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="C15">
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="E15">
         <v>50</v>
       </c>
       <c r="G15" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="B16" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="C16">
         <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="E16">
         <v>50</v>
       </c>
       <c r="G16" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="B17" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
       <c r="C17">
         <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="E17">
         <v>50</v>
       </c>
       <c r="G17" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="B18" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="C18">
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="E18">
         <v>50</v>
       </c>
       <c r="G18" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G3 A6:G7 A5:F5 A4 C4:G4 A9:G10 A8 C8:G8 A12:G13 A11 C11:G11" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:A22"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="95.796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>123</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:A22" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G3 A6:F6 A5:F5 A4 C4:G4 A9:F9 A8 C8:G8 A12:F12 A11 C11:G11 A13:F13 A10:F10 A7:F7" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>